<commit_message>
le fichier excel donne des bonne resultat final
</commit_message>
<xml_diff>
--- a/expired_domains_TLD_net.xlsx
+++ b/expired_domains_TLD_net.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -493,7 +493,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-09-29 19:41:29</t>
+          <t>2026-09-30 11:49:36</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -537,7 +537,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-09-29 19:41:29</t>
+          <t>2026-09-30 11:49:36</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -557,7 +557,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>104.21.93.65</t>
+          <t>172.67.206.42</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -572,7 +572,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>Non</t>
         </is>
       </c>
     </row>
@@ -589,7 +589,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-09-29 19:41:29</t>
+          <t>2026-09-30 11:49:36</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -633,7 +633,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-09-29 19:42:59</t>
+          <t>2026-09-30 11:50:55</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -653,7 +653,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>65.8.20.8</t>
+          <t>65.8.20.7</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -663,7 +663,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -671,6 +671,638 @@
           <t>Non</t>
         </is>
       </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Austin</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>AustinBluesRadio.com</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-09-30 11:52:14</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>AustinBluesRadio.net</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Registered</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>301</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>172.67.147.166</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Domain resolves and responds over HTTPS</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Austin</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>AustinTheArtist.com</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-09-30 11:52:14</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>AustinTheArtist.net</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Registered</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>185.230.63.107</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Domain resolves and responds over HTTPS</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Austin</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>DryCleanersAustin.com</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2026-09-30 11:52:14</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>DryCleanersAustin.net</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Registered</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>74.220.199.6</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Domain has DNS records but did not respond over HTTPS (may still be registered)</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Charlotte</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>BathroomRemodelingCharlotte.com</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-09-30 11:52:34</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>BathroomRemodelingCharlotte.net</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>No DNS record found — domain likely available or unregistered</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>San Francisco</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>SanfranciscoMotel.com</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2026-09-30 11:53:35</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>SanfranciscoMotel.net</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Registered</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>13.248.169.48</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Domain resolves and responds over HTTPS</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Las Vegas</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>LasvegasAccommodation.com</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2026-09-30 11:56:07</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>LasvegasAccommodation.net</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>No DNS record found — domain likely available or unregistered</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Memphis</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>MemphisPartyBuses.com</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2026-09-30 11:57:47</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>MemphisPartyBuses.net</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Registered</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>204.13.48.177</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Domain has DNS records but did not respond over HTTPS (may still be registered)</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Memphis</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>MemphisAnimalShelter.com</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2026-09-30 11:57:47</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>MemphisAnimalShelter.net</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Registered</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>405</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>3.33.251.168</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Domain resolves and responds over HTTPS</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Sacramento</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>WaxingSacramento.com</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2026-09-30 11:59:54</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>WaxingSacramento.net</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Registered</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>198.49.23.144</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Domain resolves and responds over HTTPS</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Miami</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>BodyShopMiami.com</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2026-09-30 12:02:14</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>BodyShopMiami.net</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Registered</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>192.185.188.169</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Domain resolves and responds over HTTPS</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Miami</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>HairExtensionMiami.com</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2026-09-30 12:02:14</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>HairExtensionMiami.net</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Registered</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>103.224.182.244</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Domain resolves and responds over HTTPS</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Bakersfield</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>GarageDoorRepairBakersfield.com</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2026-09-30 12:04:18</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>GarageDoorRepairBakersfield.net</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Registered</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>64.225.48.102</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Domain resolves and responds over HTTPS</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Tampa</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>TampaMobileDetail.com</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2026-09-30 12:05:00</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>TampaMobileDetail.net</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Registered</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>172.65.211.209</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Domain has DNS records but did not respond over HTTPS (may still be registered)</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add generated domain workbooks
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/expired_domains_TLD_net.xlsx
+++ b/expired_domains_TLD_net.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc\Desktop\DNS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18F68565-09AB-42A2-836A-C3667E16D180}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56F91DF7-62EB-4957-972D-118B38A2BD6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="93">
   <si>
     <t>City</t>
   </si>
@@ -91,9 +91,6 @@
     <t>Domain resolves and responds over HTTPS</t>
   </si>
   <si>
-    <t>9</t>
-  </si>
-  <si>
     <t>Non</t>
   </si>
   <si>
@@ -124,9 +121,6 @@
     <t>65.8.20.7</t>
   </si>
   <si>
-    <t>7</t>
-  </si>
-  <si>
     <t>Austin</t>
   </si>
   <si>
@@ -154,9 +148,6 @@
     <t>185.230.63.107</t>
   </si>
   <si>
-    <t>8</t>
-  </si>
-  <si>
     <t>DryCleanersAustin.com</t>
   </si>
   <si>
@@ -241,9 +232,6 @@
     <t>3.33.251.168</t>
   </si>
   <si>
-    <t>1</t>
-  </si>
-  <si>
     <t>Sacramento</t>
   </si>
   <si>
@@ -283,9 +271,6 @@
     <t>103.224.182.244</t>
   </si>
   <si>
-    <t>10</t>
-  </si>
-  <si>
     <t>Bakersfield</t>
   </si>
   <si>
@@ -299,9 +284,6 @@
   </si>
   <si>
     <t>64.225.48.102</t>
-  </si>
-  <si>
-    <t>2</t>
   </si>
   <si>
     <t>Tampa</t>
@@ -323,7 +305,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -331,41 +313,27 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -374,9 +342,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -684,45 +650,45 @@
   <cols>
     <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="31.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.54296875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="30.26953125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.54296875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.90625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.81640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14.453125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="69.08984375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.08984375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.26953125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
     </row>
@@ -752,36 +718,36 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+    <row r="3" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E3" t="s">
-        <v>14</v>
-      </c>
-      <c r="F3" t="s">
+      <c r="E3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H3" t="s">
+      <c r="H3" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="I3" t="s">
+      <c r="I3" s="1">
+        <v>9</v>
+      </c>
+      <c r="J3" s="1" t="s">
         <v>23</v>
-      </c>
-      <c r="J3" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
@@ -789,80 +755,80 @@
         <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C4" t="s">
         <v>12</v>
       </c>
       <c r="D4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
         <v>26</v>
       </c>
-      <c r="E4" t="s">
-        <v>14</v>
-      </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>27</v>
-      </c>
-      <c r="G4" t="s">
-        <v>28</v>
       </c>
       <c r="H4" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+    <row r="5" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G5" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E5" t="s">
-        <v>14</v>
-      </c>
-      <c r="F5" t="s">
-        <v>20</v>
-      </c>
-      <c r="G5" t="s">
-        <v>33</v>
-      </c>
-      <c r="H5" t="s">
+      <c r="H5" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="I5" t="s">
-        <v>34</v>
-      </c>
-      <c r="J5" t="s">
-        <v>24</v>
+      <c r="I5" s="1">
+        <v>7</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6" t="s">
         <v>35</v>
       </c>
-      <c r="B6" t="s">
+      <c r="D6" t="s">
         <v>36</v>
       </c>
-      <c r="C6" t="s">
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" t="s">
         <v>37</v>
       </c>
-      <c r="D6" t="s">
+      <c r="G6" t="s">
         <v>38</v>
-      </c>
-      <c r="E6" t="s">
-        <v>14</v>
-      </c>
-      <c r="F6" t="s">
-        <v>39</v>
-      </c>
-      <c r="G6" t="s">
-        <v>40</v>
       </c>
       <c r="H6" t="s">
         <v>22</v>
@@ -871,53 +837,53 @@
         <v>0</v>
       </c>
       <c r="J6" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B7" t="s">
+      <c r="D7" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G7" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C7" t="s">
-        <v>37</v>
-      </c>
-      <c r="D7" t="s">
-        <v>42</v>
-      </c>
-      <c r="E7" t="s">
-        <v>14</v>
-      </c>
-      <c r="F7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G7" t="s">
-        <v>43</v>
-      </c>
-      <c r="H7" t="s">
+      <c r="H7" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="I7" t="s">
-        <v>44</v>
-      </c>
-      <c r="J7" t="s">
-        <v>24</v>
+      <c r="I7" s="1">
+        <v>8</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
+        <v>33</v>
+      </c>
+      <c r="B8" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" t="s">
         <v>35</v>
       </c>
-      <c r="B8" t="s">
-        <v>45</v>
-      </c>
-      <c r="C8" t="s">
-        <v>37</v>
-      </c>
       <c r="D8" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="E8" t="s">
         <v>14</v>
@@ -926,7 +892,7 @@
         <v>15</v>
       </c>
       <c r="G8" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="H8" t="s">
         <v>17</v>
@@ -934,19 +900,19 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
+        <v>45</v>
+      </c>
+      <c r="B9" t="s">
+        <v>46</v>
+      </c>
+      <c r="C9" t="s">
+        <v>47</v>
+      </c>
+      <c r="D9" t="s">
         <v>48</v>
       </c>
-      <c r="B9" t="s">
+      <c r="E9" t="s">
         <v>49</v>
-      </c>
-      <c r="C9" t="s">
-        <v>50</v>
-      </c>
-      <c r="D9" t="s">
-        <v>51</v>
-      </c>
-      <c r="E9" t="s">
-        <v>52</v>
       </c>
       <c r="F9" t="s">
         <v>15</v>
@@ -955,21 +921,21 @@
         <v>15</v>
       </c>
       <c r="H9" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
+        <v>51</v>
+      </c>
+      <c r="B10" t="s">
+        <v>52</v>
+      </c>
+      <c r="C10" t="s">
+        <v>53</v>
+      </c>
+      <c r="D10" t="s">
         <v>54</v>
-      </c>
-      <c r="B10" t="s">
-        <v>55</v>
-      </c>
-      <c r="C10" t="s">
-        <v>56</v>
-      </c>
-      <c r="D10" t="s">
-        <v>57</v>
       </c>
       <c r="E10" t="s">
         <v>14</v>
@@ -978,7 +944,7 @@
         <v>20</v>
       </c>
       <c r="G10" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="H10" t="s">
         <v>22</v>
@@ -987,24 +953,24 @@
         <v>0</v>
       </c>
       <c r="J10" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
+        <v>57</v>
+      </c>
+      <c r="B11" t="s">
+        <v>58</v>
+      </c>
+      <c r="C11" t="s">
+        <v>59</v>
+      </c>
+      <c r="D11" t="s">
         <v>60</v>
       </c>
-      <c r="B11" t="s">
-        <v>61</v>
-      </c>
-      <c r="C11" t="s">
-        <v>62</v>
-      </c>
-      <c r="D11" t="s">
-        <v>63</v>
-      </c>
       <c r="E11" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="F11" t="s">
         <v>15</v>
@@ -1013,21 +979,21 @@
         <v>15</v>
       </c>
       <c r="H11" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
+        <v>61</v>
+      </c>
+      <c r="B12" t="s">
+        <v>62</v>
+      </c>
+      <c r="C12" t="s">
+        <v>63</v>
+      </c>
+      <c r="D12" t="s">
         <v>64</v>
-      </c>
-      <c r="B12" t="s">
-        <v>65</v>
-      </c>
-      <c r="C12" t="s">
-        <v>66</v>
-      </c>
-      <c r="D12" t="s">
-        <v>67</v>
       </c>
       <c r="E12" t="s">
         <v>14</v>
@@ -1036,7 +1002,7 @@
         <v>15</v>
       </c>
       <c r="G12" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="H12" t="s">
         <v>17</v>
@@ -1044,144 +1010,144 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B13" t="s">
+        <v>66</v>
+      </c>
+      <c r="C13" t="s">
+        <v>63</v>
+      </c>
+      <c r="D13" t="s">
+        <v>67</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>68</v>
+      </c>
+      <c r="G13" t="s">
         <v>69</v>
-      </c>
-      <c r="C13" t="s">
-        <v>66</v>
-      </c>
-      <c r="D13" t="s">
-        <v>70</v>
-      </c>
-      <c r="E13" t="s">
-        <v>14</v>
-      </c>
-      <c r="F13" t="s">
-        <v>71</v>
-      </c>
-      <c r="G13" t="s">
-        <v>72</v>
       </c>
       <c r="H13" t="s">
         <v>22</v>
       </c>
-      <c r="I13" t="s">
+      <c r="I13">
+        <v>1</v>
+      </c>
+      <c r="J13" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D14" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="J13" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
+      <c r="E14" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G14" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="B14" t="s">
+      <c r="H14" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I14" s="1">
+        <v>8</v>
+      </c>
+      <c r="J14" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="C14" t="s">
+      <c r="B15" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="D14" t="s">
+      <c r="C15" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="E14" t="s">
-        <v>14</v>
-      </c>
-      <c r="F14" t="s">
+      <c r="D15" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="G14" t="s">
-        <v>78</v>
-      </c>
-      <c r="H14" t="s">
+      <c r="G15" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="H15" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="I14" t="s">
-        <v>44</v>
-      </c>
-      <c r="J14" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
-        <v>79</v>
-      </c>
-      <c r="B15" t="s">
+      <c r="I15" s="1">
+        <v>9</v>
+      </c>
+      <c r="J15" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C16" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D16" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="D15" t="s">
+      <c r="E16" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G16" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="E15" t="s">
-        <v>14</v>
-      </c>
-      <c r="F15" t="s">
-        <v>20</v>
-      </c>
-      <c r="G15" t="s">
-        <v>83</v>
-      </c>
-      <c r="H15" t="s">
+      <c r="H16" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="I15" t="s">
+      <c r="I16" s="1">
+        <v>10</v>
+      </c>
+      <c r="J16" s="1" t="s">
         <v>23</v>
-      </c>
-      <c r="J15" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
-        <v>79</v>
-      </c>
-      <c r="B16" t="s">
-        <v>84</v>
-      </c>
-      <c r="C16" t="s">
-        <v>81</v>
-      </c>
-      <c r="D16" t="s">
-        <v>85</v>
-      </c>
-      <c r="E16" t="s">
-        <v>14</v>
-      </c>
-      <c r="F16" t="s">
-        <v>20</v>
-      </c>
-      <c r="G16" t="s">
-        <v>86</v>
-      </c>
-      <c r="H16" t="s">
-        <v>22</v>
-      </c>
-      <c r="I16" t="s">
-        <v>87</v>
-      </c>
-      <c r="J16" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="B17" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="C17" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="D17" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="E17" t="s">
         <v>14</v>
@@ -1190,30 +1156,30 @@
         <v>20</v>
       </c>
       <c r="G17" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="H17" t="s">
         <v>22</v>
       </c>
-      <c r="I17" t="s">
-        <v>93</v>
+      <c r="I17">
+        <v>2</v>
       </c>
       <c r="J17" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="B18" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="C18" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="D18" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="E18" t="s">
         <v>14</v>
@@ -1222,7 +1188,7 @@
         <v>15</v>
       </c>
       <c r="G18" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="H18" t="s">
         <v>17</v>

</xml_diff>